<commit_message>
anpassung beobachtungszeitraum, um stabile werte publizieren zu können
</commit_message>
<xml_diff>
--- a/KAE Ausz KonPe KTZH.xlsx
+++ b/KAE Ausz KonPe KTZH.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Werkstatt\Amtsleitung\Monitoring Covid19\Archiv Versände\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\STAT\01_Post\Schlaepfer\covid19monitoring\economy_AWA_private\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -13,7 +13,6 @@
   </bookViews>
   <sheets>
     <sheet name="März 2020" sheetId="1" r:id="rId1"/>
-    <sheet name="April 2020" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
   <si>
     <t>Metriken</t>
   </si>
@@ -118,9 +117,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>April 2020</t>
   </si>
   <si>
     <t>C 29: Fahrzeugbau</t>
@@ -147,7 +143,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -201,7 +197,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -506,13 +502,13 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -605,13 +601,13 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -627,24 +623,24 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -770,13 +766,13 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -825,7 +821,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B33">
         <v>40</v>
@@ -843,395 +839,6 @@
       </c>
       <c r="C34">
         <v>163524</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="58.5703125" customWidth="1"/>
-    <col min="2" max="2" width="39.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="3">
-        <v>75</v>
-      </c>
-      <c r="C3" s="3">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3">
-        <v>257</v>
-      </c>
-      <c r="C5" s="3">
-        <v>5219</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="3">
-        <v>123</v>
-      </c>
-      <c r="C6" s="3">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="3">
-        <v>254</v>
-      </c>
-      <c r="C7" s="3">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="3">
-        <v>43</v>
-      </c>
-      <c r="C8" s="3">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="3">
-        <v>51</v>
-      </c>
-      <c r="C9" s="3">
-        <v>695</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="3">
-        <v>173</v>
-      </c>
-      <c r="C10" s="3">
-        <v>1970</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="3">
-        <v>180</v>
-      </c>
-      <c r="C11" s="3">
-        <v>3263</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="3">
-        <v>124</v>
-      </c>
-      <c r="C12" s="3">
-        <v>2109</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="3">
-        <v>14</v>
-      </c>
-      <c r="C13" s="3">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3">
-        <v>272</v>
-      </c>
-      <c r="C14" s="3">
-        <v>2810</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>35</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="3">
-        <v>29</v>
-      </c>
-      <c r="C16" s="3">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="3">
-        <v>1186</v>
-      </c>
-      <c r="C17" s="3">
-        <v>6057</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="3">
-        <v>838</v>
-      </c>
-      <c r="C18" s="3">
-        <v>5307</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="3">
-        <v>1692</v>
-      </c>
-      <c r="C19" s="3">
-        <v>15059</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="3">
-        <v>1889</v>
-      </c>
-      <c r="C20" s="3">
-        <v>12163</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="3">
-        <v>621</v>
-      </c>
-      <c r="C21" s="3">
-        <v>18095</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="3">
-        <v>2841</v>
-      </c>
-      <c r="C22" s="3">
-        <v>30571</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="3">
-        <v>507</v>
-      </c>
-      <c r="C23" s="3">
-        <v>3440</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>22</v>
-      </c>
-      <c r="B24" s="3">
-        <v>369</v>
-      </c>
-      <c r="C24" s="3">
-        <v>1591</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>23</v>
-      </c>
-      <c r="B25" s="3">
-        <v>254</v>
-      </c>
-      <c r="C25" s="3">
-        <v>1102</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>24</v>
-      </c>
-      <c r="B26" s="3">
-        <v>3196</v>
-      </c>
-      <c r="C26" s="3">
-        <v>26744</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="3">
-        <v>1432</v>
-      </c>
-      <c r="C27" s="3">
-        <v>28421</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>36</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29" s="3">
-        <v>716</v>
-      </c>
-      <c r="C29" s="3">
-        <v>5962</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="3">
-        <v>2343</v>
-      </c>
-      <c r="C30" s="3">
-        <v>16793</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>28</v>
-      </c>
-      <c r="B31" s="3">
-        <v>778</v>
-      </c>
-      <c r="C31" s="3">
-        <v>8758</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>29</v>
-      </c>
-      <c r="B32" s="3">
-        <v>1514</v>
-      </c>
-      <c r="C32" s="3">
-        <v>7223</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33">
-        <v>21</v>
-      </c>
-      <c r="C33">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B34">
-        <v>21792</v>
-      </c>
-      <c r="C34">
-        <v>207916</v>
       </c>
     </row>
   </sheetData>

</xml_diff>